<commit_message>
Date day boards by fetch time when the header lags; re-file mislabeled boards
The hall left yesterday's date on the posted board Sun and Mon (Tue 10-20's
board was headed 10/19/26), so it was archived under the wrong day. Day boards
are now filed under max(header date, fetch-time date) with an 08:00 Pacific
cutoff, and index.json records the original header when it differs.
Also logs Thu 10-15 (day off) and Sun 10-18 (Hustler) outcomes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QU2aja5ffwwec6fCSdiUxY
</commit_message>
<xml_diff>
--- a/data/vessels/2026-10-20.xlsx
+++ b/data/vessels/2026-10-20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://portoftacoma.sharepoint.com/sites/dnateam-Technical/Shared Documents/Technical/External Dashboards/Vessel Schedule/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="441321" documentId="8_{7437B347-3B45-47A9-B5DF-E84211A5B205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBAD723E-7E39-4460-B864-5AB600294DAA}"/>
+  <xr:revisionPtr revIDLastSave="441667" documentId="8_{7437B347-3B45-47A9-B5DF-E84211A5B205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C6E43CF-0C12-4351-8694-D4AAAEEA3AC1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6E7AA7D4-05A2-4831-A105-C5B1AC660A61}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="214">
   <si>
     <t>Harbor</t>
   </si>
@@ -152,6 +152,24 @@
     <t>SSA Marine</t>
   </si>
   <si>
+    <t>WUT</t>
+  </si>
+  <si>
+    <t>PN1</t>
+  </si>
+  <si>
+    <t>YM COSMOS</t>
+  </si>
+  <si>
+    <t>PN12639W</t>
+  </si>
+  <si>
+    <t>Yang Ming</t>
+  </si>
+  <si>
+    <t>Inchcape</t>
+  </si>
+  <si>
     <t>T5</t>
   </si>
   <si>
@@ -167,24 +185,6 @@
     <t>MSC</t>
   </si>
   <si>
-    <t>WUT</t>
-  </si>
-  <si>
-    <t>PN1</t>
-  </si>
-  <si>
-    <t>YM COSMOS</t>
-  </si>
-  <si>
-    <t>PN12639W</t>
-  </si>
-  <si>
-    <t>Yang Ming</t>
-  </si>
-  <si>
-    <t>Inchcape</t>
-  </si>
-  <si>
     <t>WC4/TP5</t>
   </si>
   <si>
@@ -386,7 +386,19 @@
     <t>YM PLUM</t>
   </si>
   <si>
-    <t>PN12640W</t>
+    <t>PN12640E</t>
+  </si>
+  <si>
+    <t>LIBERTY PEACE</t>
+  </si>
+  <si>
+    <t>086S</t>
+  </si>
+  <si>
+    <t>Liberty</t>
+  </si>
+  <si>
+    <t>Pacific Terminals</t>
   </si>
   <si>
     <t>Blair</t>
@@ -395,18 +407,6 @@
     <t>LIBERTY PASSION</t>
   </si>
   <si>
-    <t>Liberty</t>
-  </si>
-  <si>
-    <t>Pacific Terminals</t>
-  </si>
-  <si>
-    <t>LIBERTY PEACE</t>
-  </si>
-  <si>
-    <t>086S</t>
-  </si>
-  <si>
     <t>FRANKFURT EXPRESS</t>
   </si>
   <si>
@@ -461,16 +461,16 @@
     <t>MC637A</t>
   </si>
   <si>
+    <t>MSC SOLA</t>
+  </si>
+  <si>
+    <t>UK643R</t>
+  </si>
+  <si>
     <t>ONE DURBAN</t>
   </si>
   <si>
-    <t>JNBB0001E</t>
-  </si>
-  <si>
-    <t>MSC SOLA</t>
-  </si>
-  <si>
-    <t>UK643R</t>
+    <t>PN32639E</t>
   </si>
   <si>
     <t>MORNING LUCY</t>
@@ -491,7 +491,7 @@
     <t>HYUNDAI FORWARD</t>
   </si>
   <si>
-    <t>HHFW0172E</t>
+    <t>PN32640W</t>
   </si>
   <si>
     <t>Not Specified</t>
@@ -500,6 +500,9 @@
     <t>CYPRESS</t>
   </si>
   <si>
+    <t>CPN0K0S19</t>
+  </si>
+  <si>
     <t>EUROPEAN HIGHWAY</t>
   </si>
   <si>
@@ -515,7 +518,7 @@
     <t>ONE MAJESTY</t>
   </si>
   <si>
-    <t>JMJT0026E</t>
+    <t>PN12641E</t>
   </si>
   <si>
     <t>EVER SMILE</t>
@@ -563,12 +566,12 @@
     <t>Jones Stevedoring Co</t>
   </si>
   <si>
+    <t>GLOVIS TREASURE</t>
+  </si>
+  <si>
     <t>GLOVIS LEGEND</t>
   </si>
   <si>
-    <t>GLOVIS TREASURE</t>
-  </si>
-  <si>
     <t>MSC SABRINA</t>
   </si>
   <si>
@@ -578,7 +581,7 @@
     <t>CORNEILLE</t>
   </si>
   <si>
-    <t>JCLL0014E</t>
+    <t>PN12642W</t>
   </si>
   <si>
     <t>WESTWOOD COLUMBIA</t>
@@ -593,7 +596,7 @@
     <t>OOCL SEATTLE</t>
   </si>
   <si>
-    <t>46E</t>
+    <t>DAH0C0E19</t>
   </si>
   <si>
     <t>COSCO SANTOS</t>
@@ -611,13 +614,16 @@
     <t>LOTUS A</t>
   </si>
   <si>
+    <t>CPN080S19</t>
+  </si>
+  <si>
     <t>GLOVIS TRUST</t>
   </si>
   <si>
     <t>ONE MODERN</t>
   </si>
   <si>
-    <t>JMOD0083E</t>
+    <t>PN32641E</t>
   </si>
   <si>
     <t>TOURMALINE ACE</t>
@@ -635,7 +641,7 @@
     <t>EVER SUMMIT</t>
   </si>
   <si>
-    <t>498-133E</t>
+    <t>NWX0E0S19</t>
   </si>
   <si>
     <t>SUPREME ACE</t>
@@ -659,22 +665,22 @@
     <t>MC639A</t>
   </si>
   <si>
+    <t>YM MANDATE</t>
+  </si>
+  <si>
+    <t>PN12643W</t>
+  </si>
+  <si>
+    <t>XIN ZHAN JIANG</t>
+  </si>
+  <si>
+    <t>201N</t>
+  </si>
+  <si>
     <t>OOCL OAKLAND</t>
   </si>
   <si>
-    <t>145E</t>
-  </si>
-  <si>
-    <t>YM MANDATE</t>
-  </si>
-  <si>
-    <t>JMDT0606E</t>
-  </si>
-  <si>
-    <t>XIN ZHAN JIANG</t>
-  </si>
-  <si>
-    <t>201N</t>
+    <t>DAH0E0E19</t>
   </si>
 </sst>
 </file>
@@ -747,10 +753,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3550F4AE-23F8-4167-8A9B-24FFB9156E08}" name="Table1" displayName="Table1" ref="A1:L108" totalsRowShown="0">
-  <autoFilter ref="A1:L108" xr:uid="{3550F4AE-23F8-4167-8A9B-24FFB9156E08}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L108">
-    <sortCondition ref="J2:J108"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3550F4AE-23F8-4167-8A9B-24FFB9156E08}" name="Table1" displayName="Table1" ref="A1:L109" totalsRowShown="0">
+  <autoFilter ref="A1:L109" xr:uid="{3550F4AE-23F8-4167-8A9B-24FFB9156E08}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L109">
+    <sortCondition ref="J2:J109"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{3ED8A004-BAC7-4959-9663-633E38656002}" name="Harbor"/>
@@ -1087,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9E2A47A-528B-46DE-AE1C-82EC550E6AFE}">
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -1281,7 +1287,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>37</v>
@@ -1299,7 +1305,7 @@
         <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
@@ -1316,25 +1322,25 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -1439,7 +1445,7 @@
         <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I10" t="s">
         <v>23</v>
@@ -1795,7 +1801,7 @@
         <v>83</v>
       </c>
       <c r="G20" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H20" t="s">
         <v>36</v>
@@ -2008,7 +2014,7 @@
         <v>21</v>
       </c>
       <c r="F26" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G26" t="s">
         <v>17</v>
@@ -2101,7 +2107,7 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C29" t="s">
         <v>98</v>
@@ -2113,10 +2119,10 @@
         <v>100</v>
       </c>
       <c r="F29" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G29" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I29" t="s">
         <v>18</v>
@@ -2235,10 +2241,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D33" t="s">
         <v>112</v>
@@ -2247,7 +2253,7 @@
         <v>113</v>
       </c>
       <c r="F33" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I33" t="s">
         <v>18</v>
@@ -2267,10 +2273,10 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D34" t="s">
         <v>114</v>
@@ -2279,10 +2285,10 @@
         <v>115</v>
       </c>
       <c r="F34" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G34" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I34" t="s">
         <v>18</v>
@@ -2302,19 +2308,22 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>116</v>
+        <v>52</v>
       </c>
       <c r="C35" t="s">
         <v>14</v>
       </c>
       <c r="D35" t="s">
+        <v>116</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>117</v>
       </c>
       <c r="F35" t="s">
         <v>118</v>
       </c>
       <c r="G35" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H35" t="s">
         <v>119</v>
@@ -2326,7 +2335,7 @@
         <v>46322.25</v>
       </c>
       <c r="K35" s="2">
-        <v>46322.75</v>
+        <v>46323.166666666664</v>
       </c>
       <c r="L35" t="s">
         <v>19</v>
@@ -2337,22 +2346,19 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>52</v>
+        <v>120</v>
       </c>
       <c r="C36" t="s">
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>120</v>
-      </c>
-      <c r="E36" s="1" t="s">
         <v>121</v>
       </c>
       <c r="F36" t="s">
         <v>118</v>
       </c>
       <c r="G36" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H36" t="s">
         <v>119</v>
@@ -2364,7 +2370,7 @@
         <v>46322.25</v>
       </c>
       <c r="K36" s="2">
-        <v>46323.166666666664</v>
+        <v>46322.75</v>
       </c>
       <c r="L36" t="s">
         <v>19</v>
@@ -2512,7 +2518,7 @@
         <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C41" t="s">
         <v>14</v>
@@ -2576,7 +2582,7 @@
         <v>31</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
         <v>129</v>
@@ -2588,7 +2594,7 @@
         <v>131</v>
       </c>
       <c r="F43" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I43" t="s">
         <v>18</v>
@@ -2701,7 +2707,7 @@
         <v>31</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C47" t="s">
         <v>129</v>
@@ -2713,7 +2719,7 @@
         <v>139</v>
       </c>
       <c r="F47" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I47" t="s">
         <v>18</v>
@@ -2768,13 +2774,13 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C49" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="D49" t="s">
         <v>140</v>
@@ -2783,7 +2789,7 @@
         <v>141</v>
       </c>
       <c r="F49" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="I49" t="s">
         <v>18</v>
@@ -2792,7 +2798,7 @@
         <v>46326.166666666664</v>
       </c>
       <c r="K49" s="2">
-        <v>46328.916666666664</v>
+        <v>46328.125</v>
       </c>
       <c r="L49" t="s">
         <v>30</v>
@@ -2800,13 +2806,13 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B50" t="s">
         <v>37</v>
       </c>
       <c r="C50" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="D50" t="s">
         <v>142</v>
@@ -2815,7 +2821,7 @@
         <v>143</v>
       </c>
       <c r="F50" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="I50" t="s">
         <v>18</v>
@@ -2824,7 +2830,7 @@
         <v>46326.166666666664</v>
       </c>
       <c r="K50" s="2">
-        <v>46328.125</v>
+        <v>46328.916666666664</v>
       </c>
       <c r="L50" t="s">
         <v>30</v>
@@ -2870,7 +2876,7 @@
         <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C52" t="s">
         <v>14</v>
@@ -2934,7 +2940,7 @@
         <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C54" t="s">
         <v>14</v>
@@ -2969,7 +2975,7 @@
         <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C55" t="s">
         <v>98</v>
@@ -3009,8 +3015,8 @@
       <c r="D56" t="s">
         <v>152</v>
       </c>
-      <c r="E56" s="1">
-        <v>70</v>
+      <c r="E56" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="F56" t="s">
         <v>106</v>
@@ -3033,16 +3039,16 @@
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C57" t="s">
         <v>14</v>
       </c>
       <c r="D57" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F57" t="s">
         <v>16</v>
@@ -3074,7 +3080,7 @@
         <v>93</v>
       </c>
       <c r="D58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E58" s="1">
         <v>2</v>
@@ -3106,7 +3112,7 @@
         <v>32</v>
       </c>
       <c r="D59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F59" t="s">
         <v>35</v>
@@ -3129,16 +3135,16 @@
         <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C60" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F60" t="s">
         <v>16</v>
@@ -3167,10 +3173,10 @@
         <v>25</v>
       </c>
       <c r="D61" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F61" t="s">
         <v>28</v>
@@ -3199,10 +3205,10 @@
         <v>14</v>
       </c>
       <c r="D62" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F62" t="s">
         <v>16</v>
@@ -3234,10 +3240,10 @@
         <v>48</v>
       </c>
       <c r="D63" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F63" t="s">
         <v>151</v>
@@ -3260,16 +3266,16 @@
         <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C64" t="s">
         <v>14</v>
       </c>
       <c r="D64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F64" t="s">
         <v>16</v>
@@ -3301,10 +3307,10 @@
         <v>93</v>
       </c>
       <c r="D65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F65" t="s">
         <v>16</v>
@@ -3333,10 +3339,10 @@
         <v>93</v>
       </c>
       <c r="D66" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F66" t="s">
         <v>16</v>
@@ -3394,10 +3400,10 @@
         <v>48</v>
       </c>
       <c r="D68" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F68" t="s">
         <v>151</v>
@@ -3426,10 +3432,10 @@
         <v>48</v>
       </c>
       <c r="D69" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F69" t="s">
         <v>151</v>
@@ -3481,19 +3487,19 @@
         <v>31</v>
       </c>
       <c r="B71" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C71" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F71" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I71" t="s">
         <v>18</v>
@@ -3519,10 +3525,10 @@
         <v>14</v>
       </c>
       <c r="D72" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F72" t="s">
         <v>56</v>
@@ -3531,7 +3537,7 @@
         <v>17</v>
       </c>
       <c r="H72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I72" t="s">
         <v>23</v>
@@ -3551,16 +3557,16 @@
         <v>12</v>
       </c>
       <c r="B73" t="s">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="C73" t="s">
         <v>14</v>
       </c>
       <c r="D73" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E73" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="s">
         <v>22</v>
@@ -3586,16 +3592,16 @@
         <v>12</v>
       </c>
       <c r="B74" t="s">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="C74" t="s">
         <v>14</v>
       </c>
       <c r="D74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E74" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F74" t="s">
         <v>22</v>
@@ -3621,19 +3627,19 @@
         <v>31</v>
       </c>
       <c r="B75" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C75" t="s">
         <v>129</v>
       </c>
       <c r="D75" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F75" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I75" t="s">
         <v>18</v>
@@ -3653,16 +3659,16 @@
         <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C76" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D76" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F76" t="s">
         <v>151</v>
@@ -3685,16 +3691,16 @@
         <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C77" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D77" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F77" t="s">
         <v>151</v>
@@ -3717,26 +3723,23 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C78" t="s">
         <v>14</v>
       </c>
       <c r="D78" t="s">
-        <v>171</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
+      </c>
+      <c r="E78" s="1">
+        <v>10</v>
       </c>
       <c r="F78" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="G78" t="s">
         <v>17</v>
       </c>
-      <c r="H78" t="s">
-        <v>173</v>
-      </c>
       <c r="I78" t="s">
         <v>23</v>
       </c>
@@ -3755,23 +3758,26 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C79" t="s">
         <v>14</v>
       </c>
       <c r="D79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E79" s="1">
-        <v>10</v>
+        <v>172</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="F79" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="G79" t="s">
         <v>17</v>
       </c>
+      <c r="H79" t="s">
+        <v>174</v>
+      </c>
       <c r="I79" t="s">
         <v>23</v>
       </c>
@@ -3796,7 +3802,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E80" s="1">
         <v>1</v>
@@ -3831,10 +3837,10 @@
         <v>75</v>
       </c>
       <c r="D81" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F81" t="s">
         <v>78</v>
@@ -3889,7 +3895,7 @@
         <v>32</v>
       </c>
       <c r="D83" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F83" t="s">
         <v>35</v>
@@ -3915,7 +3921,7 @@
         <v>32</v>
       </c>
       <c r="D84" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F84" t="s">
         <v>35</v>
@@ -3973,10 +3979,10 @@
         <v>80</v>
       </c>
       <c r="D86" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F86" t="s">
         <v>83</v>
@@ -4005,10 +4011,10 @@
         <v>107</v>
       </c>
       <c r="D87" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F87" t="s">
         <v>110</v>
@@ -4023,7 +4029,7 @@
         <v>46334</v>
       </c>
       <c r="L87" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="88" spans="1:12">
@@ -4034,10 +4040,10 @@
         <v>24</v>
       </c>
       <c r="D88" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F88" t="s">
         <v>28</v>
@@ -4095,10 +4101,10 @@
         <v>103</v>
       </c>
       <c r="D90" t="s">
-        <v>189</v>
-      </c>
-      <c r="E90" s="1">
-        <v>93</v>
+        <v>190</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="F90" t="s">
         <v>106</v>
@@ -4127,7 +4133,7 @@
         <v>14</v>
       </c>
       <c r="D91" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E91" s="1">
         <v>11</v>
@@ -4156,16 +4162,16 @@
         <v>12</v>
       </c>
       <c r="B92" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C92" t="s">
         <v>98</v>
       </c>
       <c r="D92" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F92" t="s">
         <v>16</v>
@@ -4188,16 +4194,16 @@
         <v>12</v>
       </c>
       <c r="B93" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C93" t="s">
         <v>14</v>
       </c>
       <c r="D93" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F93" t="s">
         <v>16</v>
@@ -4229,10 +4235,10 @@
         <v>14</v>
       </c>
       <c r="D94" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F94" t="s">
         <v>16</v>
@@ -4264,10 +4270,10 @@
         <v>25</v>
       </c>
       <c r="D95" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F95" t="s">
         <v>28</v>
@@ -4296,10 +4302,10 @@
         <v>25</v>
       </c>
       <c r="D96" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F96" t="s">
         <v>28</v>
@@ -4322,16 +4328,16 @@
         <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C97" t="s">
         <v>14</v>
       </c>
       <c r="D97" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F97" t="s">
         <v>16</v>
@@ -4386,19 +4392,19 @@
         <v>31</v>
       </c>
       <c r="B99" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C99" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D99" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F99" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I99" t="s">
         <v>18</v>
@@ -4453,7 +4459,7 @@
         <v>135</v>
       </c>
       <c r="D101" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F101" t="s">
         <v>78</v>
@@ -4476,19 +4482,19 @@
         <v>31</v>
       </c>
       <c r="B102" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C102" t="s">
         <v>129</v>
       </c>
       <c r="D102" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F102" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I102" t="s">
         <v>18</v>
@@ -4505,31 +4511,31 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C103" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="D103" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F103" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="I103" t="s">
         <v>18</v>
       </c>
       <c r="J103" s="2">
-        <v>46338.791666666664</v>
+        <v>46338.958333333336</v>
       </c>
       <c r="K103" s="2">
-        <v>46340.166666666664</v>
+        <v>46342.208333333336</v>
       </c>
       <c r="L103" t="s">
         <v>30</v>
@@ -4540,10 +4546,10 @@
         <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C104" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D104" t="s">
         <v>208</v>
@@ -4552,7 +4558,7 @@
         <v>209</v>
       </c>
       <c r="F104" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I104" t="s">
         <v>18</v>
@@ -4569,31 +4575,31 @@
     </row>
     <row r="105" spans="1:12">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B105" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C105" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="D105" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F105" t="s">
-        <v>46</v>
+        <v>151</v>
       </c>
       <c r="I105" t="s">
         <v>18</v>
       </c>
       <c r="J105" s="2">
-        <v>46338.958333333336</v>
+        <v>46339.083333333336</v>
       </c>
       <c r="K105" s="2">
-        <v>46342.208333333336</v>
+        <v>46340.291666666664</v>
       </c>
       <c r="L105" t="s">
         <v>30</v>
@@ -4607,25 +4613,25 @@
         <v>32</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="D106" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F106" t="s">
-        <v>151</v>
+        <v>83</v>
       </c>
       <c r="I106" t="s">
         <v>18</v>
       </c>
       <c r="J106" s="2">
-        <v>46339.083333333336</v>
+        <v>46339.291666666664</v>
       </c>
       <c r="K106" s="2">
-        <v>46340.291666666664</v>
+        <v>46340.666666666664</v>
       </c>
       <c r="L106" t="s">
         <v>30</v>
@@ -4633,28 +4639,31 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B107" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="C107" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D107" t="s">
-        <v>90</v>
+        <v>212</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>213</v>
       </c>
       <c r="F107" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="I107" t="s">
         <v>18</v>
       </c>
       <c r="J107" s="2">
-        <v>46339.541666666664</v>
+        <v>46339.291666666664</v>
       </c>
       <c r="K107" s="2">
-        <v>46340.041666666664</v>
+        <v>46340.666666666664</v>
       </c>
       <c r="L107" t="s">
         <v>30</v>
@@ -4665,27 +4674,56 @@
         <v>12</v>
       </c>
       <c r="B108" t="s">
+        <v>63</v>
+      </c>
+      <c r="C108" t="s">
+        <v>89</v>
+      </c>
+      <c r="D108" t="s">
+        <v>90</v>
+      </c>
+      <c r="F108" t="s">
+        <v>66</v>
+      </c>
+      <c r="I108" t="s">
+        <v>18</v>
+      </c>
+      <c r="J108" s="2">
+        <v>46339.541666666664</v>
+      </c>
+      <c r="K108" s="2">
+        <v>46340.041666666664</v>
+      </c>
+      <c r="L108" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12">
+      <c r="A109" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" t="s">
         <v>58</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C109" t="s">
         <v>59</v>
       </c>
-      <c r="D108" t="s">
+      <c r="D109" t="s">
         <v>91</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F109" t="s">
         <v>62</v>
       </c>
-      <c r="I108" t="s">
-        <v>18</v>
-      </c>
-      <c r="J108" s="2">
+      <c r="I109" t="s">
+        <v>18</v>
+      </c>
+      <c r="J109" s="2">
         <v>46339.704861111109</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K109" s="2">
         <v>46340.204861111109</v>
       </c>
-      <c r="L108" t="s">
+      <c r="L109" t="s">
         <v>30</v>
       </c>
     </row>
@@ -4698,12 +4736,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJ4MODS6FV673FDIUJAQKFXKCWHG:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQ01jT1hpMTlfWlJvb2tFRkZ1b1ZqbUFlYmU2eGFOY1prSzQ4ZzMwOVNrOE5z"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJYSQ36AWKC2TNDYVMQR2CLHJFKM:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQVNodndMS0ZxYlI0cXlFZENXZEpWTUFiamQ5UnJqRGdfNHFKblptMGRDaTk4"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJ4MODS6FV673FDIUJAQKFXKCWHG:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQ01jT1hpMTlfWlJvb2tFRkZ1b1ZqbUFjcU1YSmx2clY5eXMzT2hWMXFuc2ZZ"/>
+</scriptIds>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A69D21F4021FF043AD25F7555C34E75C" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ada5bbc6177f3d5462a6af737539cf89">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="169fe4b0-aa95-4062-90d3-821d069df163" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ce4529c032f5bb0135a70d700e81f25b" ns2:_="">
     <xsd:import namespace="169fe4b0-aa95-4062-90d3-821d069df163"/>
@@ -4841,7 +4887,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -4850,26 +4896,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJ4MODS6FV673FDIUJAQKFXKCWHG:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQ01jT1hpMTlfWlJvb2tFRkZ1b1ZqbUFlYmU2eGFOY1prSzQ4ZzMwOVNrOE5z"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJYSQ36AWKC2TNDYVMQR2CLHJFKM:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQVNodndMS0ZxYlI0cXlFZENXZEpWTUFiamQ5UnJqRGdfNHFKblptMGRDaTk4"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01OIHDBJ4MODS6FV673FDIUJAQKFXKCWHG:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wb3J0b2Z0YWNvbWEtbXkuc2hhcmVwb2ludC5jb20vOnU6L3AvamFsYmVyL0lRQ01jT1hpMTlfWlJvb2tFRkZ1b1ZqbUFjcU1YSmx2clY5eXMzT2hWMXFuc2ZZ"/>
-</scriptIds>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AF03C61-A585-446F-A57D-D94F9FA6CAC8}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AF8193A-09E0-4717-9CA6-EF5C70C0F2A4}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D94EB81F-BDF3-4640-AE12-B1EC3B704FEB}"/>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{090E8699-A26C-4C66-9B6D-70C00CB2CACE}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AF03C61-A585-446F-A57D-D94F9FA6CAC8}"/>
 </file>
</xml_diff>